<commit_message>
Added hyperbolic threshold sensitivity
</commit_message>
<xml_diff>
--- a/pandemic-loss-modeling/exceedance_results/bernstein_outlier.xlsx
+++ b/pandemic-loss-modeling/exceedance_results/bernstein_outlier.xlsx
@@ -393,7 +393,7 @@
         <v>0.001</v>
       </c>
       <c r="B2">
-        <v>0.9966841825751976</v>
+        <v>0.9935104121243109</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -401,7 +401,7 @@
         <v>0.002</v>
       </c>
       <c r="B3">
-        <v>0.9933893979367583</v>
+        <v>0.9871026128131208</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -409,7 +409,7 @@
         <v>7.2</v>
       </c>
       <c r="B4">
-        <v>0.03294983585893488</v>
+        <v>0.01813602799646403</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -417,7 +417,7 @@
         <v>28</v>
       </c>
       <c r="B5">
-        <v>0.007788195109246173</v>
+        <v>0.004443775412334577</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -425,7 +425,7 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>0.004669243827310834</v>
+        <v>0.002708681512121208</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -433,7 +433,7 @@
         <v>86</v>
       </c>
       <c r="B7">
-        <v>0.002316015071135645</v>
+        <v>0.001376261558283611</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -441,7 +441,7 @@
         <v>150</v>
       </c>
       <c r="B8">
-        <v>0.00126640144909073</v>
+        <v>0.0007688440662844799</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -449,7 +449,7 @@
         <v>200</v>
       </c>
       <c r="B9">
-        <v>0.0009265159999182385</v>
+        <v>0.0005688605650998471</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -457,7 +457,7 @@
         <v>220</v>
       </c>
       <c r="B10">
-        <v>0.0008353602863119923</v>
+        <v>0.0005148176373850862</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -465,7 +465,7 @@
         <v>250</v>
       </c>
       <c r="B11">
-        <v>0.0007270032859874662</v>
+        <v>0.0004503010426544003</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -473,7 +473,7 @@
         <v>280</v>
       </c>
       <c r="B12">
-        <v>0.0006427419767627664</v>
+        <v>0.0003998955314019599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>